<commit_message>
Combine rekap + Henri grades into OAK Nilai Tugas/Quiz/UTS
Filled the official Nilai Tugas, Nilai Quiz, Nilai UTS columns in each
OAK gradebook (MIK1624201 A-F, PAIK6203 A/D/E/F) by combining the TA
rekap grades with Henri's grades:
- Tugas = (tugas1*80% + tugas2*20%)*40% + tugas_henri*60%
- Kuis  = kuis*40% + kuis_henri*60%
- UTS   = uts(Sheet1, /40) + uts_henri(/60)

Sources: rekap columns in Worksheet (Tugas 01/02, Quiz), UTS in Sheet1,
Henri values from SIAP_TemplateNilai_*_Henri.xlsx (matched by NIM).
UTS left blank where the OAK Sheet1 UTS has not been entered yet
(all of class C, plus a few <75% students in other classes).
</commit_message>
<xml_diff>
--- a/nilai-oak/OAK_MIK1624201_2025_2_A.xlsx
+++ b/nilai-oak/OAK_MIK1624201_2025_2_A.xlsx
@@ -636,9 +636,15 @@
       </c>
       <c r="E8" s="3" t="n"/>
       <c r="F8" s="3" t="n"/>
-      <c r="G8" s="3" t="n"/>
-      <c r="H8" s="3" t="n"/>
-      <c r="I8" s="3" t="n"/>
+      <c r="G8" s="3" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>89.40000000000001</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>84</v>
+      </c>
       <c r="J8" s="3" t="n"/>
       <c r="K8" s="2">
         <f>ROUND( ((E8*10+F8*40+G8*10+H8*10+I8*15+J8*15) / 100), 2)</f>
@@ -683,9 +689,15 @@
       </c>
       <c r="E9" s="3" t="n"/>
       <c r="F9" s="3" t="n"/>
-      <c r="G9" s="3" t="n"/>
-      <c r="H9" s="3" t="n"/>
-      <c r="I9" s="3" t="n"/>
+      <c r="G9" s="3" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>66.40000000000001</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>65</v>
+      </c>
       <c r="J9" s="3" t="n"/>
       <c r="K9" s="2">
         <f>ROUND( ((E9*10+F9*40+G9*10+H9*10+I9*15+J9*15) / 100), 2)</f>
@@ -730,9 +742,15 @@
       </c>
       <c r="E10" s="3" t="n"/>
       <c r="F10" s="3" t="n"/>
-      <c r="G10" s="3" t="n"/>
-      <c r="H10" s="3" t="n"/>
-      <c r="I10" s="3" t="n"/>
+      <c r="G10" s="3" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>98</v>
+      </c>
       <c r="J10" s="3" t="n"/>
       <c r="K10" s="2">
         <f>ROUND( ((E10*10+F10*40+G10*10+H10*10+I10*15+J10*15) / 100), 2)</f>
@@ -777,9 +795,15 @@
       </c>
       <c r="E11" s="3" t="n"/>
       <c r="F11" s="3" t="n"/>
-      <c r="G11" s="3" t="n"/>
-      <c r="H11" s="3" t="n"/>
-      <c r="I11" s="3" t="n"/>
+      <c r="G11" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>97</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>89</v>
+      </c>
       <c r="J11" s="3" t="n"/>
       <c r="K11" s="2">
         <f>ROUND( ((E11*10+F11*40+G11*10+H11*10+I11*15+J11*15) / 100), 2)</f>
@@ -824,9 +848,15 @@
       </c>
       <c r="E12" s="3" t="n"/>
       <c r="F12" s="3" t="n"/>
-      <c r="G12" s="3" t="n"/>
-      <c r="H12" s="3" t="n"/>
-      <c r="I12" s="3" t="n"/>
+      <c r="G12" s="3" t="n">
+        <v>87</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>66</v>
+      </c>
       <c r="J12" s="3" t="n"/>
       <c r="K12" s="2">
         <f>ROUND( ((E12*10+F12*40+G12*10+H12*10+I12*15+J12*15) / 100), 2)</f>
@@ -871,9 +901,15 @@
       </c>
       <c r="E13" s="3" t="n"/>
       <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-      <c r="H13" s="3" t="n"/>
-      <c r="I13" s="3" t="n"/>
+      <c r="G13" s="3" t="n">
+        <v>83.59999999999999</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>93</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>57</v>
+      </c>
       <c r="J13" s="3" t="n"/>
       <c r="K13" s="2">
         <f>ROUND( ((E13*10+F13*40+G13*10+H13*10+I13*15+J13*15) / 100), 2)</f>
@@ -918,9 +954,15 @@
       </c>
       <c r="E14" s="3" t="n"/>
       <c r="F14" s="3" t="n"/>
-      <c r="G14" s="3" t="n"/>
-      <c r="H14" s="3" t="n"/>
-      <c r="I14" s="3" t="n"/>
+      <c r="G14" s="3" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>90.2</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>84</v>
+      </c>
       <c r="J14" s="3" t="n"/>
       <c r="K14" s="2">
         <f>ROUND( ((E14*10+F14*40+G14*10+H14*10+I14*15+J14*15) / 100), 2)</f>
@@ -965,9 +1007,15 @@
       </c>
       <c r="E15" s="3" t="n"/>
       <c r="F15" s="3" t="n"/>
-      <c r="G15" s="3" t="n"/>
-      <c r="H15" s="3" t="n"/>
-      <c r="I15" s="3" t="n"/>
+      <c r="G15" s="3" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>78</v>
+      </c>
       <c r="J15" s="3" t="n"/>
       <c r="K15" s="2">
         <f>ROUND( ((E15*10+F15*40+G15*10+H15*10+I15*15+J15*15) / 100), 2)</f>
@@ -1012,9 +1060,15 @@
       </c>
       <c r="E16" s="3" t="n"/>
       <c r="F16" s="3" t="n"/>
-      <c r="G16" s="3" t="n"/>
-      <c r="H16" s="3" t="n"/>
-      <c r="I16" s="3" t="n"/>
+      <c r="G16" s="3" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>83</v>
+      </c>
       <c r="J16" s="3" t="n"/>
       <c r="K16" s="2">
         <f>ROUND( ((E16*10+F16*40+G16*10+H16*10+I16*15+J16*15) / 100), 2)</f>
@@ -1059,9 +1113,15 @@
       </c>
       <c r="E17" s="3" t="n"/>
       <c r="F17" s="3" t="n"/>
-      <c r="G17" s="3" t="n"/>
-      <c r="H17" s="3" t="n"/>
-      <c r="I17" s="3" t="n"/>
+      <c r="G17" s="3" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>71</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>78</v>
+      </c>
       <c r="J17" s="3" t="n"/>
       <c r="K17" s="2">
         <f>ROUND( ((E17*10+F17*40+G17*10+H17*10+I17*15+J17*15) / 100), 2)</f>
@@ -1106,9 +1166,15 @@
       </c>
       <c r="E18" s="3" t="n"/>
       <c r="F18" s="3" t="n"/>
-      <c r="G18" s="3" t="n"/>
-      <c r="H18" s="3" t="n"/>
-      <c r="I18" s="3" t="n"/>
+      <c r="G18" s="3" t="n">
+        <v>82.8</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>86.59999999999999</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>84</v>
+      </c>
       <c r="J18" s="3" t="n"/>
       <c r="K18" s="2">
         <f>ROUND( ((E18*10+F18*40+G18*10+H18*10+I18*15+J18*15) / 100), 2)</f>
@@ -1153,9 +1219,15 @@
       </c>
       <c r="E19" s="3" t="n"/>
       <c r="F19" s="3" t="n"/>
-      <c r="G19" s="3" t="n"/>
-      <c r="H19" s="3" t="n"/>
-      <c r="I19" s="3" t="n"/>
+      <c r="G19" s="3" t="n">
+        <v>70.2</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>69.40000000000001</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>80</v>
+      </c>
       <c r="J19" s="3" t="n"/>
       <c r="K19" s="2">
         <f>ROUND( ((E19*10+F19*40+G19*10+H19*10+I19*15+J19*15) / 100), 2)</f>
@@ -1200,9 +1272,15 @@
       </c>
       <c r="E20" s="3" t="n"/>
       <c r="F20" s="3" t="n"/>
-      <c r="G20" s="3" t="n"/>
-      <c r="H20" s="3" t="n"/>
-      <c r="I20" s="3" t="n"/>
+      <c r="G20" s="3" t="n">
+        <v>84</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>86</v>
+      </c>
       <c r="J20" s="3" t="n"/>
       <c r="K20" s="2">
         <f>ROUND( ((E20*10+F20*40+G20*10+H20*10+I20*15+J20*15) / 100), 2)</f>
@@ -1247,9 +1325,15 @@
       </c>
       <c r="E21" s="3" t="n"/>
       <c r="F21" s="3" t="n"/>
-      <c r="G21" s="3" t="n"/>
-      <c r="H21" s="3" t="n"/>
-      <c r="I21" s="3" t="n"/>
+      <c r="G21" s="3" t="n">
+        <v>79.59999999999999</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>64</v>
+      </c>
       <c r="J21" s="3" t="n"/>
       <c r="K21" s="2">
         <f>ROUND( ((E21*10+F21*40+G21*10+H21*10+I21*15+J21*15) / 100), 2)</f>
@@ -1294,9 +1378,15 @@
       </c>
       <c r="E22" s="3" t="n"/>
       <c r="F22" s="3" t="n"/>
-      <c r="G22" s="3" t="n"/>
-      <c r="H22" s="3" t="n"/>
-      <c r="I22" s="3" t="n"/>
+      <c r="G22" s="3" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="J22" s="3" t="n"/>
       <c r="K22" s="2">
         <f>ROUND( ((E22*10+F22*40+G22*10+H22*10+I22*15+J22*15) / 100), 2)</f>
@@ -1341,9 +1431,15 @@
       </c>
       <c r="E23" s="3" t="n"/>
       <c r="F23" s="3" t="n"/>
-      <c r="G23" s="3" t="n"/>
-      <c r="H23" s="3" t="n"/>
-      <c r="I23" s="3" t="n"/>
+      <c r="G23" s="3" t="n">
+        <v>86.2</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>82</v>
+      </c>
       <c r="J23" s="3" t="n"/>
       <c r="K23" s="2">
         <f>ROUND( ((E23*10+F23*40+G23*10+H23*10+I23*15+J23*15) / 100), 2)</f>
@@ -1388,9 +1484,15 @@
       </c>
       <c r="E24" s="3" t="n"/>
       <c r="F24" s="3" t="n"/>
-      <c r="G24" s="3" t="n"/>
-      <c r="H24" s="3" t="n"/>
-      <c r="I24" s="3" t="n"/>
+      <c r="G24" s="3" t="n">
+        <v>79.2</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>77</v>
+      </c>
       <c r="J24" s="3" t="n"/>
       <c r="K24" s="2">
         <f>ROUND( ((E24*10+F24*40+G24*10+H24*10+I24*15+J24*15) / 100), 2)</f>
@@ -1435,9 +1537,15 @@
       </c>
       <c r="E25" s="3" t="n"/>
       <c r="F25" s="3" t="n"/>
-      <c r="G25" s="3" t="n"/>
-      <c r="H25" s="3" t="n"/>
-      <c r="I25" s="3" t="n"/>
+      <c r="G25" s="3" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>62</v>
+      </c>
       <c r="J25" s="3" t="n"/>
       <c r="K25" s="2">
         <f>ROUND( ((E25*10+F25*40+G25*10+H25*10+I25*15+J25*15) / 100), 2)</f>
@@ -1482,9 +1590,15 @@
       </c>
       <c r="E26" s="3" t="n"/>
       <c r="F26" s="3" t="n"/>
-      <c r="G26" s="3" t="n"/>
-      <c r="H26" s="3" t="n"/>
-      <c r="I26" s="3" t="n"/>
+      <c r="G26" s="3" t="n">
+        <v>80.2</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>86.8</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>40</v>
+      </c>
       <c r="J26" s="3" t="n"/>
       <c r="K26" s="2">
         <f>ROUND( ((E26*10+F26*40+G26*10+H26*10+I26*15+J26*15) / 100), 2)</f>
@@ -1529,9 +1643,15 @@
       </c>
       <c r="E27" s="3" t="n"/>
       <c r="F27" s="3" t="n"/>
-      <c r="G27" s="3" t="n"/>
-      <c r="H27" s="3" t="n"/>
-      <c r="I27" s="3" t="n"/>
+      <c r="G27" s="3" t="n">
+        <v>75.8</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>91.2</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>70</v>
+      </c>
       <c r="J27" s="3" t="n"/>
       <c r="K27" s="2">
         <f>ROUND( ((E27*10+F27*40+G27*10+H27*10+I27*15+J27*15) / 100), 2)</f>
@@ -1576,9 +1696,15 @@
       </c>
       <c r="E28" s="3" t="n"/>
       <c r="F28" s="3" t="n"/>
-      <c r="G28" s="3" t="n"/>
-      <c r="H28" s="3" t="n"/>
-      <c r="I28" s="3" t="n"/>
+      <c r="G28" s="3" t="n">
+        <v>76.2</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>59</v>
+      </c>
       <c r="J28" s="3" t="n"/>
       <c r="K28" s="2">
         <f>ROUND( ((E28*10+F28*40+G28*10+H28*10+I28*15+J28*15) / 100), 2)</f>
@@ -1623,9 +1749,15 @@
       </c>
       <c r="E29" s="3" t="n"/>
       <c r="F29" s="3" t="n"/>
-      <c r="G29" s="3" t="n"/>
-      <c r="H29" s="3" t="n"/>
-      <c r="I29" s="3" t="n"/>
+      <c r="G29" s="3" t="n">
+        <v>82.59999999999999</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>55.2</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>17</v>
+      </c>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="2">
         <f>ROUND( ((E29*10+F29*40+G29*10+H29*10+I29*15+J29*15) / 100), 2)</f>
@@ -1670,9 +1802,15 @@
       </c>
       <c r="E30" s="3" t="n"/>
       <c r="F30" s="3" t="n"/>
-      <c r="G30" s="3" t="n"/>
-      <c r="H30" s="3" t="n"/>
-      <c r="I30" s="3" t="n"/>
+      <c r="G30" s="3" t="n">
+        <v>76</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>88.8</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>78</v>
+      </c>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="2">
         <f>ROUND( ((E30*10+F30*40+G30*10+H30*10+I30*15+J30*15) / 100), 2)</f>
@@ -1717,9 +1855,15 @@
       </c>
       <c r="E31" s="3" t="n"/>
       <c r="F31" s="3" t="n"/>
-      <c r="G31" s="3" t="n"/>
-      <c r="H31" s="3" t="n"/>
-      <c r="I31" s="3" t="n"/>
+      <c r="G31" s="3" t="n">
+        <v>84.40000000000001</v>
+      </c>
+      <c r="H31" s="3" t="n">
+        <v>96.40000000000001</v>
+      </c>
+      <c r="I31" s="3" t="n">
+        <v>51</v>
+      </c>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="2">
         <f>ROUND( ((E31*10+F31*40+G31*10+H31*10+I31*15+J31*15) / 100), 2)</f>
@@ -1764,9 +1908,15 @@
       </c>
       <c r="E32" s="3" t="n"/>
       <c r="F32" s="3" t="n"/>
-      <c r="G32" s="3" t="n"/>
-      <c r="H32" s="3" t="n"/>
-      <c r="I32" s="3" t="n"/>
+      <c r="G32" s="3" t="n">
+        <v>85</v>
+      </c>
+      <c r="H32" s="3" t="n">
+        <v>91.8</v>
+      </c>
+      <c r="I32" s="3" t="n">
+        <v>54</v>
+      </c>
       <c r="J32" s="3" t="n"/>
       <c r="K32" s="2">
         <f>ROUND( ((E32*10+F32*40+G32*10+H32*10+I32*15+J32*15) / 100), 2)</f>
@@ -1811,9 +1961,15 @@
       </c>
       <c r="E33" s="3" t="n"/>
       <c r="F33" s="3" t="n"/>
-      <c r="G33" s="3" t="n"/>
-      <c r="H33" s="3" t="n"/>
-      <c r="I33" s="3" t="n"/>
+      <c r="G33" s="3" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="H33" s="3" t="n">
+        <v>74</v>
+      </c>
+      <c r="I33" s="3" t="n">
+        <v>77</v>
+      </c>
       <c r="J33" s="3" t="n"/>
       <c r="K33" s="2">
         <f>ROUND( ((E33*10+F33*40+G33*10+H33*10+I33*15+J33*15) / 100), 2)</f>
@@ -1858,9 +2014,15 @@
       </c>
       <c r="E34" s="3" t="n"/>
       <c r="F34" s="3" t="n"/>
-      <c r="G34" s="3" t="n"/>
-      <c r="H34" s="3" t="n"/>
-      <c r="I34" s="3" t="n"/>
+      <c r="G34" s="3" t="n">
+        <v>83</v>
+      </c>
+      <c r="H34" s="3" t="n">
+        <v>80.40000000000001</v>
+      </c>
+      <c r="I34" s="3" t="n">
+        <v>44</v>
+      </c>
       <c r="J34" s="3" t="n"/>
       <c r="K34" s="2">
         <f>ROUND( ((E34*10+F34*40+G34*10+H34*10+I34*15+J34*15) / 100), 2)</f>
@@ -1905,9 +2067,15 @@
       </c>
       <c r="E35" s="3" t="n"/>
       <c r="F35" s="3" t="n"/>
-      <c r="G35" s="3" t="n"/>
-      <c r="H35" s="3" t="n"/>
-      <c r="I35" s="3" t="n"/>
+      <c r="G35" s="3" t="n">
+        <v>84.2</v>
+      </c>
+      <c r="H35" s="3" t="n">
+        <v>55.8</v>
+      </c>
+      <c r="I35" s="3" t="n">
+        <v>49</v>
+      </c>
       <c r="J35" s="3" t="n"/>
       <c r="K35" s="2">
         <f>ROUND( ((E35*10+F35*40+G35*10+H35*10+I35*15+J35*15) / 100), 2)</f>
@@ -1952,9 +2120,15 @@
       </c>
       <c r="E36" s="3" t="n"/>
       <c r="F36" s="3" t="n"/>
-      <c r="G36" s="3" t="n"/>
-      <c r="H36" s="3" t="n"/>
-      <c r="I36" s="3" t="n"/>
+      <c r="G36" s="3" t="n">
+        <v>83.8</v>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="I36" s="3" t="n">
+        <v>48</v>
+      </c>
       <c r="J36" s="3" t="n"/>
       <c r="K36" s="2">
         <f>ROUND( ((E36*10+F36*40+G36*10+H36*10+I36*15+J36*15) / 100), 2)</f>
@@ -1999,9 +2173,15 @@
       </c>
       <c r="E37" s="3" t="n"/>
       <c r="F37" s="3" t="n"/>
-      <c r="G37" s="3" t="n"/>
-      <c r="H37" s="3" t="n"/>
-      <c r="I37" s="3" t="n"/>
+      <c r="G37" s="3" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>86</v>
+      </c>
+      <c r="I37" s="3" t="n">
+        <v>71</v>
+      </c>
       <c r="J37" s="3" t="n"/>
       <c r="K37" s="2">
         <f>ROUND( ((E37*10+F37*40+G37*10+H37*10+I37*15+J37*15) / 100), 2)</f>
@@ -2046,9 +2226,15 @@
       </c>
       <c r="E38" s="3" t="n"/>
       <c r="F38" s="3" t="n"/>
-      <c r="G38" s="3" t="n"/>
-      <c r="H38" s="3" t="n"/>
-      <c r="I38" s="3" t="n"/>
+      <c r="G38" s="3" t="n">
+        <v>73.59999999999999</v>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>68.8</v>
+      </c>
+      <c r="I38" s="3" t="n">
+        <v>76</v>
+      </c>
       <c r="J38" s="3" t="n"/>
       <c r="K38" s="2">
         <f>ROUND( ((E38*10+F38*40+G38*10+H38*10+I38*15+J38*15) / 100), 2)</f>
@@ -2093,9 +2279,15 @@
       </c>
       <c r="E39" s="3" t="n"/>
       <c r="F39" s="3" t="n"/>
-      <c r="G39" s="3" t="n"/>
-      <c r="H39" s="3" t="n"/>
-      <c r="I39" s="3" t="n"/>
+      <c r="G39" s="3" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>87.8</v>
+      </c>
+      <c r="I39" s="3" t="n">
+        <v>70</v>
+      </c>
       <c r="J39" s="3" t="n"/>
       <c r="K39" s="2">
         <f>ROUND( ((E39*10+F39*40+G39*10+H39*10+I39*15+J39*15) / 100), 2)</f>
@@ -2140,9 +2332,15 @@
       </c>
       <c r="E40" s="3" t="n"/>
       <c r="F40" s="3" t="n"/>
-      <c r="G40" s="3" t="n"/>
-      <c r="H40" s="3" t="n"/>
-      <c r="I40" s="3" t="n"/>
+      <c r="G40" s="3" t="n">
+        <v>84.59999999999999</v>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="I40" s="3" t="n">
+        <v>76</v>
+      </c>
       <c r="J40" s="3" t="n"/>
       <c r="K40" s="2">
         <f>ROUND( ((E40*10+F40*40+G40*10+H40*10+I40*15+J40*15) / 100), 2)</f>
@@ -2187,9 +2385,15 @@
       </c>
       <c r="E41" s="3" t="n"/>
       <c r="F41" s="3" t="n"/>
-      <c r="G41" s="3" t="n"/>
-      <c r="H41" s="3" t="n"/>
-      <c r="I41" s="3" t="n"/>
+      <c r="G41" s="3" t="n">
+        <v>77</v>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>85.40000000000001</v>
+      </c>
+      <c r="I41" s="3" t="n">
+        <v>15</v>
+      </c>
       <c r="J41" s="3" t="n"/>
       <c r="K41" s="2">
         <f>ROUND( ((E41*10+F41*40+G41*10+H41*10+I41*15+J41*15) / 100), 2)</f>
@@ -2234,9 +2438,15 @@
       </c>
       <c r="E42" s="3" t="n"/>
       <c r="F42" s="3" t="n"/>
-      <c r="G42" s="3" t="n"/>
-      <c r="H42" s="3" t="n"/>
-      <c r="I42" s="3" t="n"/>
+      <c r="G42" s="3" t="n">
+        <v>82.40000000000001</v>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>89</v>
+      </c>
+      <c r="I42" s="3" t="n">
+        <v>47</v>
+      </c>
       <c r="J42" s="3" t="n"/>
       <c r="K42" s="2">
         <f>ROUND( ((E42*10+F42*40+G42*10+H42*10+I42*15+J42*15) / 100), 2)</f>
@@ -2281,9 +2491,15 @@
       </c>
       <c r="E43" s="3" t="n"/>
       <c r="F43" s="3" t="n"/>
-      <c r="G43" s="3" t="n"/>
-      <c r="H43" s="3" t="n"/>
-      <c r="I43" s="3" t="n"/>
+      <c r="G43" s="3" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>88.40000000000001</v>
+      </c>
+      <c r="I43" s="3" t="n">
+        <v>78</v>
+      </c>
       <c r="J43" s="3" t="n"/>
       <c r="K43" s="2">
         <f>ROUND( ((E43*10+F43*40+G43*10+H43*10+I43*15+J43*15) / 100), 2)</f>
@@ -2328,9 +2544,15 @@
       </c>
       <c r="E44" s="3" t="n"/>
       <c r="F44" s="3" t="n"/>
-      <c r="G44" s="3" t="n"/>
-      <c r="H44" s="3" t="n"/>
-      <c r="I44" s="3" t="n"/>
+      <c r="G44" s="3" t="n">
+        <v>82.2</v>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>66.2</v>
+      </c>
+      <c r="I44" s="3" t="n">
+        <v>20</v>
+      </c>
       <c r="J44" s="3" t="n"/>
       <c r="K44" s="2">
         <f>ROUND( ((E44*10+F44*40+G44*10+H44*10+I44*15+J44*15) / 100), 2)</f>
@@ -2375,9 +2597,15 @@
       </c>
       <c r="E45" s="3" t="n"/>
       <c r="F45" s="3" t="n"/>
-      <c r="G45" s="3" t="n"/>
-      <c r="H45" s="3" t="n"/>
-      <c r="I45" s="3" t="n"/>
+      <c r="G45" s="3" t="n">
+        <v>74.59999999999999</v>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>71.2</v>
+      </c>
+      <c r="I45" s="3" t="n">
+        <v>77</v>
+      </c>
       <c r="J45" s="3" t="n"/>
       <c r="K45" s="2">
         <f>ROUND( ((E45*10+F45*40+G45*10+H45*10+I45*15+J45*15) / 100), 2)</f>
@@ -2422,9 +2650,15 @@
       </c>
       <c r="E46" s="3" t="n"/>
       <c r="F46" s="3" t="n"/>
-      <c r="G46" s="3" t="n"/>
-      <c r="H46" s="3" t="n"/>
-      <c r="I46" s="3" t="n"/>
+      <c r="G46" s="3" t="n">
+        <v>85.2</v>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>84.8</v>
+      </c>
+      <c r="I46" s="3" t="n">
+        <v>43</v>
+      </c>
       <c r="J46" s="3" t="n"/>
       <c r="K46" s="2">
         <f>ROUND( ((E46*10+F46*40+G46*10+H46*10+I46*15+J46*15) / 100), 2)</f>

</xml_diff>